<commit_message>
Added apparent shunt and deadspace ratio outputs that use blood gas values instead of fluid mechanics properties. Improved respiratory system compliance calculations. Updated ventilator validation scenarios. Updated mainstem intubation scenario for better validation.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator/MechanicalVentilator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Programming\Pulse\engine\data\human\adult\validation\Scenarios\MechanicalVentilator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\MechanicalVentilator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24CEE40-7404-4AFB-B968-1781631DEA88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D10258-0E2E-40EE-A702-6050782588DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="23250" yWindow="6450" windowWidth="28365" windowHeight="21600" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="COPD" sheetId="13" r:id="rId3"/>
     <sheet name="Recruitment" sheetId="14" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="815" uniqueCount="190">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -206,9 +206,6 @@
 }</t>
   </si>
   <si>
-    <t>ShuntFraction</t>
-  </si>
-  <si>
     <t>MechanicalVentilatorHealthy</t>
   </si>
   <si>
@@ -289,9 +286,6 @@
     }</t>
   </si>
   <si>
-    <t>PhysiologicDeadSpaceTidalVolumeRatio</t>
-  </si>
-  <si>
     <t>VD/VT</t>
   </si>
   <si>
@@ -314,12 +308,6 @@
   </si>
   <si>
     <t>QS/QT</t>
-  </si>
-  <si>
-    <t>QS/QT (0.33 +/- 0.15)</t>
-  </si>
-  <si>
-    <t>QS/QT (0.22 +/- 0.14)</t>
   </si>
   <si>
     <t>PaO2/FiO2</t>
@@ -789,6 +777,36 @@
   </si>
   <si>
     <t>{v} = 438</t>
+  </si>
+  <si>
+    <t>ApparentShuntFraction</t>
+  </si>
+  <si>
+    <t>ApparentPhysiologicDeadSpaceTidalVolumeRatio</t>
+  </si>
+  <si>
+    <t>Good:0, Fair:10</t>
+  </si>
+  <si>
+    <t>Good:0, Fair:2</t>
+  </si>
+  <si>
+    <t>ShuntFraction</t>
+  </si>
+  <si>
+    <t>PhysiologicDeadSpaceTidalVolumeRatio</t>
+  </si>
+  <si>
+    <t>VD/VT (determined from blood gas values)</t>
+  </si>
+  <si>
+    <t>QS/QT (determined from blood gas values)</t>
+  </si>
+  <si>
+    <t>QS/QT (determined from blood gas values) (0.33 +/- 0.15)</t>
+  </si>
+  <si>
+    <t>QS/QT (determined from blood gas values) (0.22 +/- 0.14)</t>
   </si>
 </sst>
 </file>
@@ -1051,12 +1069,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1077,6 +1089,12 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1473,7 +1491,7 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="11" customWidth="1"/>
-    <col min="2" max="2" width="36.28515625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="48.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="11" customWidth="1"/>
     <col min="4" max="4" width="25" style="11" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" style="11" customWidth="1"/>
@@ -1504,16 +1522,16 @@
     </row>
     <row r="2" spans="1:8" ht="177.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
       <c r="E2" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20"/>
@@ -1540,11 +1558,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -1568,7 +1586,7 @@
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="17" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H5" s="17"/>
     </row>
@@ -1577,60 +1595,60 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="24"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="28"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1642,13 +1660,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9" t="s">
         <v>20</v>
@@ -1658,13 +1676,13 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="9"/>
       <c r="H12" s="9"/>
     </row>
@@ -1672,15 +1690,15 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+      <c r="B13" s="28" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="9" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H13" s="9"/>
     </row>
@@ -1688,13 +1706,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
+      <c r="B14" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -1709,13 +1727,13 @@
         <v>11</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>6</v>
@@ -1735,10 +1753,10 @@
         <v>34</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F16" s="10"/>
       <c r="G16" s="12" t="s">
@@ -1757,10 +1775,10 @@
         <v>34</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F17" s="10"/>
       <c r="G17" s="12" t="s">
@@ -1779,10 +1797,10 @@
         <v>33</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="12" t="s">
@@ -1795,20 +1813,20 @@
         <v>23</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>68</v>
+        <v>185</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="12" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -1817,20 +1835,20 @@
         <v>23</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>50</v>
+        <v>184</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -1845,14 +1863,14 @@
         <v>36</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F21" s="10"/>
       <c r="G21" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -1867,12 +1885,14 @@
         <v>25</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F22" s="10"/>
+        <v>123</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G22" s="12" t="s">
         <v>41</v>
       </c>
@@ -1889,10 +1909,10 @@
         <v>28</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="2" t="s">
@@ -1911,10 +1931,10 @@
         <v>28</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F24" s="10"/>
       <c r="G24" s="2" t="s">
@@ -1933,10 +1953,10 @@
         <v>25</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F25" s="10"/>
       <c r="G25" s="2" t="s">
@@ -1955,14 +1975,16 @@
         <v>28</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F26" s="10"/>
+        <v>123</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G26" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H26" s="16"/>
     </row>
@@ -1977,14 +1999,14 @@
         <v>28</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H27" s="16"/>
     </row>
@@ -2027,7 +2049,7 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="11" customWidth="1"/>
-    <col min="2" max="2" width="36.28515625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="48.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="11" customWidth="1"/>
     <col min="4" max="4" width="25" style="11" customWidth="1"/>
     <col min="5" max="5" width="39" style="11" customWidth="1"/>
@@ -2058,16 +2080,16 @@
     </row>
     <row r="2" spans="1:8" ht="241.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
       <c r="E2" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20"/>
@@ -2094,11 +2116,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -2122,7 +2144,7 @@
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="17" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H5" s="17"/>
     </row>
@@ -2131,60 +2153,60 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="24"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="28"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -2210,15 +2232,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
+      <c r="B12" s="28" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -2226,13 +2248,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -2242,13 +2264,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -2256,15 +2278,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
+      <c r="B15" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -2272,13 +2294,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
+      <c r="B16" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -2293,13 +2315,13 @@
         <v>11</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>6</v>
@@ -2319,10 +2341,10 @@
         <v>34</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="12" t="s">
@@ -2341,10 +2363,10 @@
         <v>34</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="12" t="s">
@@ -2363,10 +2385,10 @@
         <v>33</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="12" t="s">
@@ -2379,20 +2401,20 @@
         <v>23</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F21" s="10"/>
       <c r="G21" s="12" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -2401,20 +2423,20 @@
         <v>23</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -2429,14 +2451,14 @@
         <v>36</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H23" s="16"/>
     </row>
@@ -2451,12 +2473,14 @@
         <v>25</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F24" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="G24" s="12" t="s">
         <v>41</v>
       </c>
@@ -2473,12 +2497,14 @@
         <v>28</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F25" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G25" s="2" t="s">
         <v>43</v>
       </c>
@@ -2495,12 +2521,14 @@
         <v>28</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F26" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G26" s="2" t="s">
         <v>42</v>
       </c>
@@ -2517,12 +2545,14 @@
         <v>25</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G27" s="2" t="s">
         <v>44</v>
       </c>
@@ -2539,14 +2569,16 @@
         <v>28</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F28" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G28" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -2561,14 +2593,16 @@
         <v>28</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="F29" s="10"/>
+        <v>119</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G29" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H29" s="16"/>
     </row>
@@ -2576,13 +2610,13 @@
       <c r="A30" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="29"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
       <c r="G30" s="1" t="s">
         <v>6</v>
       </c>
@@ -2594,15 +2628,15 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
+      <c r="B31" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
       <c r="G31" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H31" s="9"/>
     </row>
@@ -2610,15 +2644,15 @@
       <c r="A32" s="8">
         <v>2</v>
       </c>
-      <c r="B32" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21"/>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
+      <c r="B32" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" s="28"/>
+      <c r="D32" s="28"/>
+      <c r="E32" s="28"/>
+      <c r="F32" s="28"/>
       <c r="G32" s="9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H32" s="9"/>
     </row>
@@ -2626,13 +2660,13 @@
       <c r="A33" s="8">
         <v>2</v>
       </c>
-      <c r="B33" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
+      <c r="B33" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C33" s="28"/>
+      <c r="D33" s="28"/>
+      <c r="E33" s="28"/>
+      <c r="F33" s="28"/>
       <c r="G33" s="9"/>
       <c r="H33" s="9"/>
     </row>
@@ -2647,13 +2681,13 @@
         <v>11</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>6</v>
@@ -2673,10 +2707,10 @@
         <v>34</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F35" s="10"/>
       <c r="G35" s="12" t="s">
@@ -2695,10 +2729,10 @@
         <v>34</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F36" s="10"/>
       <c r="G36" s="12" t="s">
@@ -2717,10 +2751,10 @@
         <v>33</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F37" s="10"/>
       <c r="G37" s="12" t="s">
@@ -2733,20 +2767,20 @@
         <v>23</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="12" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="H38" s="16"/>
     </row>
@@ -2755,20 +2789,20 @@
         <v>23</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F39" s="10"/>
       <c r="G39" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H39" s="16"/>
     </row>
@@ -2783,14 +2817,14 @@
         <v>36</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F40" s="10"/>
       <c r="G40" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H40" s="16"/>
     </row>
@@ -2805,12 +2839,14 @@
         <v>25</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F41" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="G41" s="12" t="s">
         <v>41</v>
       </c>
@@ -2827,12 +2863,14 @@
         <v>28</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F42" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G42" s="2" t="s">
         <v>43</v>
       </c>
@@ -2849,12 +2887,14 @@
         <v>28</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F43" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F43" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G43" s="2" t="s">
         <v>42</v>
       </c>
@@ -2871,12 +2911,14 @@
         <v>25</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F44" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="F44" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G44" s="2" t="s">
         <v>44</v>
       </c>
@@ -2893,14 +2935,16 @@
         <v>28</v>
       </c>
       <c r="D45" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F45" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G45" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H45" s="16"/>
     </row>
@@ -2915,14 +2959,16 @@
         <v>28</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="F46" s="10"/>
+        <v>119</v>
+      </c>
+      <c r="F46" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G46" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H46" s="16"/>
     </row>
@@ -2930,13 +2976,13 @@
       <c r="A47" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B47" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
-      <c r="F47" s="29"/>
+      <c r="C47" s="27"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
+      <c r="F47" s="27"/>
       <c r="G47" s="1" t="s">
         <v>6</v>
       </c>
@@ -2948,15 +2994,15 @@
       <c r="A48" s="8">
         <v>3</v>
       </c>
-      <c r="B48" s="21" t="s">
+      <c r="B48" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C48" s="21"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
+      <c r="C48" s="28"/>
+      <c r="D48" s="28"/>
+      <c r="E48" s="28"/>
+      <c r="F48" s="28"/>
       <c r="G48" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="H48" s="9"/>
     </row>
@@ -2964,15 +3010,15 @@
       <c r="A49" s="8">
         <v>3</v>
       </c>
-      <c r="B49" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C49" s="21"/>
-      <c r="D49" s="21"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="21"/>
+      <c r="B49" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="C49" s="28"/>
+      <c r="D49" s="28"/>
+      <c r="E49" s="28"/>
+      <c r="F49" s="28"/>
       <c r="G49" s="9" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="H49" s="9"/>
     </row>
@@ -2980,13 +3026,13 @@
       <c r="A50" s="8">
         <v>3</v>
       </c>
-      <c r="B50" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C50" s="21"/>
-      <c r="D50" s="21"/>
-      <c r="E50" s="21"/>
-      <c r="F50" s="21"/>
+      <c r="B50" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="28"/>
+      <c r="D50" s="28"/>
+      <c r="E50" s="28"/>
+      <c r="F50" s="28"/>
       <c r="G50" s="9"/>
       <c r="H50" s="9"/>
     </row>
@@ -3001,13 +3047,13 @@
         <v>11</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>6</v>
@@ -3027,10 +3073,10 @@
         <v>34</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F52" s="10"/>
       <c r="G52" s="12" t="s">
@@ -3049,10 +3095,10 @@
         <v>34</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F53" s="10"/>
       <c r="G53" s="12" t="s">
@@ -3071,10 +3117,10 @@
         <v>33</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F54" s="10"/>
       <c r="G54" s="12" t="s">
@@ -3087,20 +3133,20 @@
         <v>23</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="C55" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F55" s="10"/>
       <c r="G55" s="12" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="H55" s="16"/>
     </row>
@@ -3109,20 +3155,20 @@
         <v>23</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C56" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F56" s="10"/>
       <c r="G56" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H56" s="16"/>
     </row>
@@ -3137,14 +3183,14 @@
         <v>36</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F57" s="10"/>
       <c r="G57" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H57" s="16"/>
     </row>
@@ -3159,12 +3205,14 @@
         <v>25</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F58" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F58" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="G58" s="12" t="s">
         <v>41</v>
       </c>
@@ -3181,12 +3229,14 @@
         <v>28</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F59" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F59" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G59" s="2" t="s">
         <v>43</v>
       </c>
@@ -3203,12 +3253,14 @@
         <v>28</v>
       </c>
       <c r="D60" s="2" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F60" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F60" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G60" s="2" t="s">
         <v>42</v>
       </c>
@@ -3225,12 +3277,14 @@
         <v>25</v>
       </c>
       <c r="D61" s="2" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F61" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="F61" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G61" s="2" t="s">
         <v>44</v>
       </c>
@@ -3247,14 +3301,16 @@
         <v>28</v>
       </c>
       <c r="D62" s="2" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E62" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F62" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F62" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G62" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H62" s="16"/>
     </row>
@@ -3269,14 +3325,14 @@
         <v>28</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E63" s="10" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F63" s="10"/>
       <c r="G63" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H63" s="16"/>
     </row>
@@ -3328,7 +3384,7 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="11" customWidth="1"/>
-    <col min="2" max="2" width="36.28515625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="48.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="11" customWidth="1"/>
     <col min="4" max="4" width="25" style="11" customWidth="1"/>
     <col min="5" max="5" width="39.28515625" style="11" customWidth="1"/>
@@ -3359,16 +3415,16 @@
     </row>
     <row r="2" spans="1:8" ht="283.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
       <c r="E2" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20"/>
@@ -3395,11 +3451,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -3423,7 +3479,7 @@
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="17" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H5" s="17"/>
     </row>
@@ -3432,60 +3488,60 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="24"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="28"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -3497,13 +3553,13 @@
       <c r="A11" s="8">
         <v>1</v>
       </c>
-      <c r="B11" s="21" t="s">
+      <c r="B11" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
       <c r="G11" s="9"/>
       <c r="H11" s="9"/>
     </row>
@@ -3511,15 +3567,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="21" t="s">
+      <c r="B12" s="28" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -3527,13 +3583,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -3543,13 +3599,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -3557,15 +3613,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
+      <c r="B15" s="28" t="s">
+        <v>130</v>
+      </c>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -3573,13 +3629,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
+      <c r="B16" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -3594,13 +3650,13 @@
         <v>11</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>6</v>
@@ -3620,10 +3676,10 @@
         <v>34</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="12" t="s">
@@ -3642,10 +3698,10 @@
         <v>34</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F19" s="10"/>
       <c r="G19" s="12" t="s">
@@ -3664,10 +3720,10 @@
         <v>33</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F20" s="10"/>
       <c r="G20" s="12" t="s">
@@ -3680,20 +3736,20 @@
         <v>23</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F21" s="10"/>
       <c r="G21" s="12" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="H21" s="16"/>
     </row>
@@ -3702,20 +3758,20 @@
         <v>23</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F22" s="10"/>
       <c r="G22" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H22" s="16"/>
     </row>
@@ -3730,14 +3786,14 @@
         <v>36</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F23" s="10"/>
       <c r="G23" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H23" s="16"/>
     </row>
@@ -3752,12 +3808,14 @@
         <v>25</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F24" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="G24" s="12" t="s">
         <v>41</v>
       </c>
@@ -3774,12 +3832,14 @@
         <v>28</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F25" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G25" s="2" t="s">
         <v>43</v>
       </c>
@@ -3796,12 +3856,14 @@
         <v>28</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F26" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G26" s="2" t="s">
         <v>42</v>
       </c>
@@ -3818,12 +3880,14 @@
         <v>25</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G27" s="2" t="s">
         <v>44</v>
       </c>
@@ -3833,13 +3897,13 @@
       <c r="A28" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="29"/>
+      <c r="C28" s="27"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
       <c r="G28" s="1" t="s">
         <v>6</v>
       </c>
@@ -3851,15 +3915,15 @@
       <c r="A29" s="8">
         <v>2</v>
       </c>
-      <c r="B29" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="F29" s="21"/>
+      <c r="B29" s="28" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+      <c r="F29" s="28"/>
       <c r="G29" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="H29" s="9"/>
     </row>
@@ -3868,14 +3932,14 @@
         <v>2</v>
       </c>
       <c r="B30" s="30" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C30" s="31"/>
       <c r="D30" s="31"/>
       <c r="E30" s="31"/>
       <c r="F30" s="32"/>
       <c r="G30" s="9" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="H30" s="9"/>
     </row>
@@ -3883,13 +3947,13 @@
       <c r="A31" s="8">
         <v>2</v>
       </c>
-      <c r="B31" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C31" s="21"/>
-      <c r="D31" s="21"/>
-      <c r="E31" s="21"/>
-      <c r="F31" s="21"/>
+      <c r="B31" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
+      <c r="F31" s="28"/>
       <c r="G31" s="9"/>
       <c r="H31" s="9"/>
     </row>
@@ -3904,13 +3968,13 @@
         <v>11</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>6</v>
@@ -3930,10 +3994,10 @@
         <v>34</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F33" s="10"/>
       <c r="G33" s="12" t="s">
@@ -3952,10 +4016,10 @@
         <v>34</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F34" s="10"/>
       <c r="G34" s="12" t="s">
@@ -3974,10 +4038,10 @@
         <v>33</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F35" s="10"/>
       <c r="G35" s="12" t="s">
@@ -3990,20 +4054,20 @@
         <v>23</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F36" s="10"/>
       <c r="G36" s="12" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="H36" s="16"/>
     </row>
@@ -4012,20 +4076,20 @@
         <v>23</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F37" s="10"/>
       <c r="G37" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H37" s="16"/>
     </row>
@@ -4040,14 +4104,14 @@
         <v>36</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F38" s="10"/>
       <c r="G38" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H38" s="16"/>
     </row>
@@ -4062,12 +4126,14 @@
         <v>25</v>
       </c>
       <c r="D39" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F39" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="G39" s="12" t="s">
         <v>41</v>
       </c>
@@ -4084,12 +4150,14 @@
         <v>28</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F40" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G40" s="2" t="s">
         <v>43</v>
       </c>
@@ -4106,12 +4174,14 @@
         <v>28</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F41" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G41" s="2" t="s">
         <v>42</v>
       </c>
@@ -4128,12 +4198,14 @@
         <v>25</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F42" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="F42" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G42" s="2" t="s">
         <v>44</v>
       </c>
@@ -4143,13 +4215,13 @@
       <c r="A43" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B43" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
+      <c r="C43" s="27"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="27"/>
+      <c r="F43" s="27"/>
       <c r="G43" s="1" t="s">
         <v>6</v>
       </c>
@@ -4161,15 +4233,15 @@
       <c r="A44" s="8">
         <v>3</v>
       </c>
-      <c r="B44" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C44" s="21"/>
-      <c r="D44" s="21"/>
-      <c r="E44" s="21"/>
-      <c r="F44" s="21"/>
+      <c r="B44" s="28" t="s">
+        <v>66</v>
+      </c>
+      <c r="C44" s="28"/>
+      <c r="D44" s="28"/>
+      <c r="E44" s="28"/>
+      <c r="F44" s="28"/>
       <c r="G44" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H44" s="9"/>
     </row>
@@ -4178,14 +4250,14 @@
         <v>3</v>
       </c>
       <c r="B45" s="30" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C45" s="31"/>
       <c r="D45" s="31"/>
       <c r="E45" s="31"/>
       <c r="F45" s="32"/>
       <c r="G45" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="H45" s="9"/>
     </row>
@@ -4193,13 +4265,13 @@
       <c r="A46" s="8">
         <v>3</v>
       </c>
-      <c r="B46" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
+      <c r="B46" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C46" s="28"/>
+      <c r="D46" s="28"/>
+      <c r="E46" s="28"/>
+      <c r="F46" s="28"/>
       <c r="G46" s="9"/>
       <c r="H46" s="9"/>
     </row>
@@ -4214,13 +4286,13 @@
         <v>11</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>6</v>
@@ -4240,10 +4312,10 @@
         <v>34</v>
       </c>
       <c r="D48" s="2" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E48" s="10" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F48" s="10"/>
       <c r="G48" s="12" t="s">
@@ -4262,10 +4334,10 @@
         <v>34</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="F49" s="10"/>
       <c r="G49" s="12" t="s">
@@ -4284,10 +4356,10 @@
         <v>33</v>
       </c>
       <c r="D50" s="2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F50" s="10"/>
       <c r="G50" s="12" t="s">
@@ -4300,20 +4372,20 @@
         <v>23</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>68</v>
+        <v>181</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D51" s="2" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="F51" s="10"/>
       <c r="G51" s="12" t="s">
-        <v>69</v>
+        <v>186</v>
       </c>
       <c r="H51" s="16"/>
     </row>
@@ -4322,20 +4394,20 @@
         <v>23</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C52" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D52" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F52" s="10"/>
       <c r="G52" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H52" s="16"/>
     </row>
@@ -4350,14 +4422,14 @@
         <v>36</v>
       </c>
       <c r="D53" s="2" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="F53" s="10"/>
       <c r="G53" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H53" s="16"/>
     </row>
@@ -4372,12 +4444,14 @@
         <v>25</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F54" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>183</v>
+      </c>
       <c r="G54" s="12" t="s">
         <v>41</v>
       </c>
@@ -4394,12 +4468,14 @@
         <v>28</v>
       </c>
       <c r="D55" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F55" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F55" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G55" s="2" t="s">
         <v>43</v>
       </c>
@@ -4416,12 +4492,14 @@
         <v>28</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="F56" s="10"/>
+        <v>75</v>
+      </c>
+      <c r="F56" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G56" s="2" t="s">
         <v>42</v>
       </c>
@@ -4438,12 +4516,14 @@
         <v>25</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F57" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="F57" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G57" s="2" t="s">
         <v>44</v>
       </c>
@@ -4497,7 +4577,7 @@
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24.85546875" style="11" customWidth="1"/>
-    <col min="2" max="2" width="36.28515625" style="11" customWidth="1"/>
+    <col min="2" max="2" width="35.7109375" style="11" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="11" customWidth="1"/>
     <col min="4" max="4" width="25" style="11" customWidth="1"/>
     <col min="5" max="5" width="35.5703125" style="11" customWidth="1"/>
@@ -4528,16 +4608,16 @@
     </row>
     <row r="2" spans="1:8" ht="82.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
       <c r="D2" s="19"/>
       <c r="E2" s="4" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="G2" s="20"/>
       <c r="H2" s="20"/>
@@ -4564,11 +4644,11 @@
       <c r="A4" s="7">
         <v>0</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
       <c r="G4" s="3"/>
       <c r="H4" s="16" t="s">
         <v>8</v>
@@ -4592,7 +4672,7 @@
       </c>
       <c r="F5" s="17"/>
       <c r="G5" s="17" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="H5" s="17"/>
     </row>
@@ -4601,60 +4681,60 @@
       <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="7"/>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
-      <c r="H6" s="24"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="15"/>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
       <c r="D7" s="7"/>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
+      <c r="F7" s="29"/>
+      <c r="G7" s="23"/>
+      <c r="H7" s="24"/>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15"/>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
       <c r="D8" s="7"/>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="23"/>
+      <c r="H8" s="24"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="7"/>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="F9" s="22"/>
-      <c r="G9" s="27"/>
-      <c r="H9" s="28"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26"/>
     </row>
     <row r="10" spans="1:8" ht="14.85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
+      <c r="C10" s="27"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="27"/>
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
@@ -4680,15 +4760,15 @@
       <c r="A12" s="8">
         <v>1</v>
       </c>
-      <c r="B12" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
+      <c r="B12" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
+      <c r="E12" s="28"/>
+      <c r="F12" s="28"/>
       <c r="G12" s="9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="H12" s="9"/>
     </row>
@@ -4696,13 +4776,13 @@
       <c r="A13" s="8">
         <v>1</v>
       </c>
-      <c r="B13" s="21" t="s">
+      <c r="B13" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="28"/>
       <c r="G13" s="9"/>
       <c r="H13" s="9" t="s">
         <v>20</v>
@@ -4712,13 +4792,13 @@
       <c r="A14" s="8">
         <v>1</v>
       </c>
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
       <c r="G14" s="9"/>
       <c r="H14" s="9"/>
     </row>
@@ -4726,15 +4806,15 @@
       <c r="A15" s="8">
         <v>1</v>
       </c>
-      <c r="B15" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
+      <c r="B15" s="28" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
       <c r="G15" s="9" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="H15" s="9"/>
     </row>
@@ -4742,13 +4822,13 @@
       <c r="A16" s="8">
         <v>1</v>
       </c>
-      <c r="B16" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
+      <c r="B16" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="28"/>
+      <c r="F16" s="28"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
@@ -4763,13 +4843,13 @@
         <v>11</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>6</v>
@@ -4789,14 +4869,14 @@
         <v>36</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F18" s="10"/>
       <c r="G18" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H18" s="16"/>
     </row>
@@ -4811,14 +4891,16 @@
         <v>28</v>
       </c>
       <c r="D19" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F19" s="10"/>
+      <c r="F19" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G19" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="H19" s="16"/>
     </row>
@@ -4827,20 +4909,22 @@
         <v>23</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F20" s="10"/>
+        <v>61</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G20" s="2" t="s">
-        <v>76</v>
+        <v>188</v>
       </c>
       <c r="H20" s="16"/>
     </row>
@@ -4848,13 +4932,13 @@
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="29" t="s">
+      <c r="B21" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="29"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
       <c r="G21" s="1" t="s">
         <v>6</v>
       </c>
@@ -4866,15 +4950,15 @@
       <c r="A22" s="8">
         <v>2</v>
       </c>
-      <c r="B22" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
+      <c r="B22" s="28" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" s="28"/>
+      <c r="D22" s="28"/>
+      <c r="E22" s="28"/>
+      <c r="F22" s="28"/>
       <c r="G22" s="9" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H22" s="9"/>
     </row>
@@ -4882,13 +4966,13 @@
       <c r="A23" s="8">
         <v>2</v>
       </c>
-      <c r="B23" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C23" s="21"/>
-      <c r="D23" s="21"/>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
+      <c r="B23" s="28" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="28"/>
+      <c r="D23" s="28"/>
+      <c r="E23" s="28"/>
+      <c r="F23" s="28"/>
       <c r="G23" s="9"/>
       <c r="H23" s="9"/>
     </row>
@@ -4903,13 +4987,13 @@
         <v>11</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>6</v>
@@ -4929,14 +5013,14 @@
         <v>36</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F25" s="10"/>
       <c r="G25" s="2" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="H25" s="16"/>
     </row>
@@ -4951,10 +5035,10 @@
         <v>28</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F26" s="10"/>
       <c r="G26" s="2" t="s">
@@ -4973,10 +5057,10 @@
         <v>28</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F27" s="10"/>
       <c r="G27" s="2" t="s">
@@ -4995,14 +5079,16 @@
         <v>28</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F28" s="10"/>
+        <v>61</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G28" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="H28" s="16"/>
     </row>
@@ -5017,14 +5103,14 @@
         <v>28</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F29" s="10"/>
       <c r="G29" s="2" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H29" s="16"/>
     </row>
@@ -5033,20 +5119,22 @@
         <v>23</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="F30" s="10"/>
+        <v>61</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>182</v>
+      </c>
       <c r="G30" s="2" t="s">
-        <v>77</v>
+        <v>189</v>
       </c>
       <c r="H30" s="16"/>
     </row>
@@ -5055,20 +5143,20 @@
         <v>23</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F31" s="10"/>
       <c r="G31" s="2" t="s">
-        <v>75</v>
+        <v>187</v>
       </c>
       <c r="H31" s="16"/>
     </row>

</xml_diff>

<commit_message>
Mechanical ventilator validation calibration updates.
</commit_message>
<xml_diff>
--- a/data/human/adult/validation/Scenarios/MechanicalVentilator/MechanicalVentilator.xlsx
+++ b/data/human/adult/validation/Scenarios/MechanicalVentilator/MechanicalVentilator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\Source\Pulse\ventilator_scenarios\source\data\human\adult\validation\Scenarios\MechanicalVentilator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84D10258-0E2E-40EE-A702-6050782588DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{282BEA5A-4BF1-4BDD-A694-8076EAE081CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23250" yWindow="6450" windowWidth="28365" windowHeight="21600" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2175" yWindow="5085" windowWidth="26580" windowHeight="25920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Healthy" sheetId="15" r:id="rId1"/>

</xml_diff>